<commit_message>
CDD-013: normalize authority release artifacts
</commit_message>
<xml_diff>
--- a/architecture/released/v1.4/RELEASE-MANIFEST-v1.4.xlsx
+++ b/architecture/released/v1.4/RELEASE-MANIFEST-v1.4.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="Rc37d1624146848b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="R56bd2cd0b99d4c22"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -451,7 +451,7 @@
         <x:v>AUTHORITATIVE</x:v>
       </x:c>
       <x:c r="H7" s="11" t="str">
-        <x:v>61a43bd33ea381fed75533547fb25b02b348e2c947e966de923fad5107b42d0b</x:v>
+        <x:v>d4afeb07180512636fc7352823bcdc4c11fd7a649be6dac751925f9f04e8ee89</x:v>
       </x:c>
       <x:c r="I7" s="11" t="str"/>
       <x:c r="J7" s="11" t="str">
@@ -481,7 +481,7 @@
         <x:v>AUTHORITATIVE</x:v>
       </x:c>
       <x:c r="H8" s="11" t="str">
-        <x:v>9a9a118dfd1fefccf8c705e354d453151823d3991c4c6e6fcffbdd36eb187afc</x:v>
+        <x:v>0e5e0fa03e31a7c7eaff61e39910e33449d2fe2f3c0e9586113f0201b61f0531</x:v>
       </x:c>
       <x:c r="I8" s="11" t="str"/>
       <x:c r="J8" s="11" t="str">
@@ -511,7 +511,7 @@
         <x:v>AUTHORITATIVE</x:v>
       </x:c>
       <x:c r="H9" s="11" t="str">
-        <x:v>dcbc4da3384357a3c1e66c302e51ad708166a0f7ab6dfd69b1bbdaf99079c9b7</x:v>
+        <x:v>56501a1814dfdd23c9aba51353f624fbc7a6db96279d76dd04bda602016587a2</x:v>
       </x:c>
       <x:c r="I9" s="11" t="str">
         <x:v>RFC-014 v1.2</x:v>
@@ -543,7 +543,7 @@
         <x:v>AUTHORITATIVE</x:v>
       </x:c>
       <x:c r="H10" s="11" t="str">
-        <x:v>e9f328840b907db8c75c474a9f573a7915aec84a5e9c64d1627cfcdaa978d6d4</x:v>
+        <x:v>fbd0f6d520b2e28bd306ac502117e271ea82a65936796a8cdc9a4a69a0a5da5d</x:v>
       </x:c>
       <x:c r="I10" s="11" t="str">
         <x:v>PMM-001 v1.1</x:v>
@@ -607,7 +607,7 @@
         <x:v>AUTHORITATIVE</x:v>
       </x:c>
       <x:c r="H12" s="11" t="str">
-        <x:v>7557bb2ee1fe20a180cf75f49cd2f6b2cd27c13b71337672ce2bbf2e3dff0765</x:v>
+        <x:v>4f96a5cea077bc5a0ccf1a11bfc56309eb1fe9357a7e68fd0e8beff2ad30bb0b</x:v>
       </x:c>
       <x:c r="I12" s="11" t="str">
         <x:v>Architecture Dependency Matrix v1.3</x:v>
@@ -639,7 +639,7 @@
         <x:v>AUTHORITATIVE</x:v>
       </x:c>
       <x:c r="H13" s="11" t="str">
-        <x:v>d6d5b475f0914ae309c81c88cfcc2bb549ada16d6dadaa9cf372038eb72026e9</x:v>
+        <x:v>1197a1c42bb93193c84acdc3a4cdf59056cc9f503f82b30aa1328259b4349bc3</x:v>
       </x:c>
       <x:c r="I13" s="11" t="str">
         <x:v>Baseline Record v1.5</x:v>
@@ -671,7 +671,7 @@
         <x:v>AUTHORITATIVE</x:v>
       </x:c>
       <x:c r="H14" s="11" t="str">
-        <x:v>dd80f4a7d39772e359f1d4932b5cf43249472c99221b77c49db1ee9152cbec3b</x:v>
+        <x:v>dd40662ebd37984fe05b5c1b392b96438c23430d4930255ab2ff8b9000b5f6d2</x:v>
       </x:c>
       <x:c r="I14" s="11" t="str">
         <x:v>ACR-001 v1.4</x:v>
@@ -703,7 +703,7 @@
         <x:v>AUTHORITATIVE</x:v>
       </x:c>
       <x:c r="H15" s="11" t="str">
-        <x:v>31c1cccd90cc51ecd0acda442d8d0723f07590525a14725e704632164867095e</x:v>
+        <x:v>10c798f004e63fdf1a6184658fc4bf697d258a65954961f26e83d8d6db22e8ae</x:v>
       </x:c>
       <x:c r="I15" s="11" t="str">
         <x:v>ADR-001 v1.4</x:v>
@@ -735,7 +735,7 @@
         <x:v>AUTHORITATIVE</x:v>
       </x:c>
       <x:c r="H16" s="11" t="str">
-        <x:v>4303fe20faba55892903bd70c02dc6f0bf67e08216b575db4a37754a07a74a36</x:v>
+        <x:v>ac88e5f1d3e4af5ffe28946d47c8521d2359d0afaf873e989c1f5cc1028aab8a</x:v>
       </x:c>
       <x:c r="I16" s="11" t="str">
         <x:v>RRR-001 v1.4</x:v>

</xml_diff>